<commit_message>
Release v1.0.3: BodyText Hinweis bei Zusatzanhaengen
</commit_message>
<xml_diff>
--- a/data/Auswahl Teilnehmende zu Lernbereichen.xlsx
+++ b/data/Auswahl Teilnehmende zu Lernbereichen.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Git-Projekte INN-tegrativ gGmbH\Themenlisten-Helfer\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/746d0da4b5755b4d/Git-Projekte INN-tegrativ gGmbH/Themenlisten-Helfer/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4C8B3FF-5E8B-4F06-8EAD-8B58095200E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{D4C8B3FF-5E8B-4F06-8EAD-8B58095200E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8182F231-7973-4267-BB9A-18DFEE1406C9}"/>
   <bookViews>
     <workbookView xWindow="2490" yWindow="1530" windowWidth="26310" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="266">
   <si>
     <t>Anrede</t>
   </si>
@@ -834,6 +834,9 @@
   </si>
   <si>
     <t>Terveer, Andrea</t>
+  </si>
+  <si>
+    <t>Lehmkuhl_KLR_Arbeitsmaterial.pdf</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1009,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2937,7 +2942,9 @@
       <c r="C9" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="D9" s="22"/>
+      <c r="D9" s="22" t="s">
+        <v>265</v>
+      </c>
       <c r="E9" s="22"/>
       <c r="F9" s="22"/>
       <c r="G9" s="22"/>

</xml_diff>

<commit_message>
feat(data): update participant selection and template documents
</commit_message>
<xml_diff>
--- a/data/Auswahl Teilnehmende zu Lernbereichen.xlsx
+++ b/data/Auswahl Teilnehmende zu Lernbereichen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/746d0da4b5755b4d/Git-Projekte INN-tegrativ gGmbH/Themenlisten-Helfer/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\12. WE\QUA\C1 KFM-Verw\K-Team\Team\__Team - Tools\Themenlisten-Helfer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{D4C8B3FF-5E8B-4F06-8EAD-8B58095200E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8182F231-7973-4267-BB9A-18DFEE1406C9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBF05BA-8F7E-44F4-A6DE-E7BC1301ECBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2490" yWindow="1530" windowWidth="26310" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teilnehmende" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Hilfstabellen" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Teilnehmende!$A$1:$G$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Teilnehmende!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,12 +34,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="242">
   <si>
     <t>Anrede</t>
   </si>
@@ -68,135 +71,24 @@
     <t>Herr</t>
   </si>
   <si>
-    <t>Marc William</t>
-  </si>
-  <si>
-    <t>Evers</t>
-  </si>
-  <si>
-    <t>11.05. - 05.06.2026</t>
-  </si>
-  <si>
-    <t>KBM 2506</t>
-  </si>
-  <si>
     <t>Assistenz und Sekretariat</t>
   </si>
   <si>
     <t>Nein</t>
   </si>
   <si>
-    <t>Jordan Bouke</t>
-  </si>
-  <si>
-    <t>Fluitman</t>
-  </si>
-  <si>
-    <t>Steffen</t>
-  </si>
-  <si>
-    <t>Grummel</t>
-  </si>
-  <si>
-    <t>Pasquale</t>
-  </si>
-  <si>
-    <t>Guida</t>
-  </si>
-  <si>
     <t>Marketing und Vertrieb</t>
   </si>
   <si>
     <t>Frau</t>
   </si>
   <si>
-    <t>Sonja</t>
-  </si>
-  <si>
-    <t>Kalyta</t>
-  </si>
-  <si>
     <t>Manuela</t>
   </si>
   <si>
-    <t>Kirmes</t>
-  </si>
-  <si>
     <t>Maik</t>
   </si>
   <si>
-    <t>Mücke</t>
-  </si>
-  <si>
-    <t>Marco</t>
-  </si>
-  <si>
-    <t>Ockenga</t>
-  </si>
-  <si>
-    <t>Nicole</t>
-  </si>
-  <si>
-    <t>Sandkötter</t>
-  </si>
-  <si>
-    <t>Michelle Louisa</t>
-  </si>
-  <si>
-    <t>Seefeldt</t>
-  </si>
-  <si>
-    <t>Katharina</t>
-  </si>
-  <si>
-    <t>Simke</t>
-  </si>
-  <si>
-    <t>Gustav</t>
-  </si>
-  <si>
-    <t>Stoll</t>
-  </si>
-  <si>
-    <t>Monika</t>
-  </si>
-  <si>
-    <t>Süßmuth</t>
-  </si>
-  <si>
-    <t>Dennis</t>
-  </si>
-  <si>
-    <t>Thiems</t>
-  </si>
-  <si>
-    <t>Matthias</t>
-  </si>
-  <si>
-    <t>Hugen</t>
-  </si>
-  <si>
-    <t>BFK 2506</t>
-  </si>
-  <si>
-    <t>Christina</t>
-  </si>
-  <si>
-    <t>Duhm</t>
-  </si>
-  <si>
-    <t>Selma</t>
-  </si>
-  <si>
-    <t>Seldüz</t>
-  </si>
-  <si>
-    <t>Anne-Dörte</t>
-  </si>
-  <si>
-    <t>Tangemann</t>
-  </si>
-  <si>
     <t>Julia</t>
   </si>
   <si>
@@ -377,12 +269,6 @@
     <t>Yannik</t>
   </si>
   <si>
-    <t>Marineße</t>
-  </si>
-  <si>
-    <t>Loreen</t>
-  </si>
-  <si>
     <t>Meinke</t>
   </si>
   <si>
@@ -401,12 +287,6 @@
     <t>Reeck</t>
   </si>
   <si>
-    <t>Riethmüller</t>
-  </si>
-  <si>
-    <t>Darron</t>
-  </si>
-  <si>
     <t>Sasse</t>
   </si>
   <si>
@@ -626,9 +506,6 @@
     <t>Lange, Yannik</t>
   </si>
   <si>
-    <t>Marineße, Loreen</t>
-  </si>
-  <si>
     <t>Meinke, Jannyn</t>
   </si>
   <si>
@@ -641,9 +518,6 @@
     <t>Reeck, Torsten</t>
   </si>
   <si>
-    <t>Riethmüller, Darron</t>
-  </si>
-  <si>
     <t>Sasse, Corinna</t>
   </si>
   <si>
@@ -677,9 +551,6 @@
     <t>Bönsch, Julia</t>
   </si>
   <si>
-    <t>Busko, Nico</t>
-  </si>
-  <si>
     <t>Christians, Yvonne</t>
   </si>
   <si>
@@ -837,13 +708,73 @@
   </si>
   <si>
     <t>Lehmkuhl_KLR_Arbeitsmaterial.pdf</t>
+  </si>
+  <si>
+    <t>Behrends, Benjamin</t>
+  </si>
+  <si>
+    <t>Hoffmann, Tobias</t>
+  </si>
+  <si>
+    <t>Klar-Janssen, Markus</t>
+  </si>
+  <si>
+    <t>Linnemann, Kristin</t>
+  </si>
+  <si>
+    <t>Mraw, Mohamed</t>
+  </si>
+  <si>
+    <t>Rosen, Jennifer</t>
+  </si>
+  <si>
+    <t>Zimmermann, Lara</t>
+  </si>
+  <si>
+    <t>Behrends</t>
+  </si>
+  <si>
+    <t>Benjamin</t>
+  </si>
+  <si>
+    <t>Hoffmann</t>
+  </si>
+  <si>
+    <t>Klar-Janssen</t>
+  </si>
+  <si>
+    <t>Markus</t>
+  </si>
+  <si>
+    <t>Linnemann</t>
+  </si>
+  <si>
+    <t>Kristin</t>
+  </si>
+  <si>
+    <t>Mraw</t>
+  </si>
+  <si>
+    <t>Mohamed</t>
+  </si>
+  <si>
+    <t>Rosen</t>
+  </si>
+  <si>
+    <t>Lara</t>
+  </si>
+  <si>
+    <t>06.07. - 28.08.2026</t>
+  </si>
+  <si>
+    <t>Ja</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -868,6 +799,11 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -956,7 +892,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1004,9 +940,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
@@ -1380,7 +1313,7 @@
   <sheetPr codeName="Tabelle1">
     <tabColor theme="9" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.28515625" customWidth="1"/>
@@ -1413,150 +1346,150 @@
       <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="21">
-        <f>COUNTIF($G$2:$G$40,"Ja")</f>
-        <v>0</v>
+      <c r="J1" s="20">
+        <f>COUNTIF($G$2:$G$100,"Ja")</f>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>14</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>14</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>143</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>21</v>
+        <v>144</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>14</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>21</v>
+        <v>143</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>14</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -1564,160 +1497,160 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>29</v>
+      <c r="B9" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>21</v>
+        <v>141</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>21</v>
+        <v>143</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>21</v>
+        <v>143</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>21</v>
+        <v>144</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>14</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -1725,1043 +1658,787 @@
         <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>13</v>
+        <v>143</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>21</v>
+        <v>141</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>21</v>
+        <v>141</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>21</v>
+        <v>141</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>55</v>
+        <v>143</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>58</v>
+        <v>141</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>61</v>
+        <v>144</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>14</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>63</v>
+        <v>8</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>230</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>229</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>65</v>
+      <c r="B24" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>93</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>95</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>67</v>
+        <v>12</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>62</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>71</v>
+      <c r="C27" s="19" t="s">
+        <v>67</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>72</v>
+        <v>240</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>55</v>
+        <v>142</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>74</v>
+        <v>8</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>69</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>76</v>
+        <v>12</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>78</v>
+      <c r="B30" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>231</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>80</v>
+        <v>8</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>232</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>61</v>
+        <v>142</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>82</v>
+        <v>8</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>73</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>84</v>
+        <v>12</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>234</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>61</v>
+        <v>142</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>86</v>
+        <v>12</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>75</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>88</v>
+        <v>12</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>236</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>58</v>
+        <v>142</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>90</v>
+        <v>12</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>77</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>92</v>
+        <v>12</v>
+      </c>
+      <c r="B37" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>96</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>95</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>94</v>
+        <v>8</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="19" t="s">
+        <v>79</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E38" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>61</v>
+        <v>142</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>96</v>
+      <c r="B39" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="19" t="s">
+        <v>80</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E39" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>55</v>
+        <v>142</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>98</v>
+        <v>12</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>238</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>54</v>
+        <v>240</v>
+      </c>
+      <c r="E40" s="19" t="s">
+        <v>64</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>61</v>
+        <v>142</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F41" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="G41" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F42" s="20"/>
+        <v>95</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="G42" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B43" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>105</v>
+        <v>12</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F43" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="G43" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B44" s="19" t="s">
-        <v>106</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>107</v>
+      <c r="B44" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F44" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="G44" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B45" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>109</v>
+        <v>12</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F45" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="G45" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B46" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>111</v>
+        <v>12</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F46" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="G46" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B47" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="C47" s="19" t="s">
-        <v>113</v>
+        <v>12</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F47" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>142</v>
+      </c>
       <c r="G47" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>115</v>
+        <v>12</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>11</v>
+        <v>240</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F48" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="G48" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B49" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F49" s="20"/>
-      <c r="G49" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B50" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C50" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F50" s="20"/>
-      <c r="G50" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="C51" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F51" s="20"/>
-      <c r="G51" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F52" s="20"/>
-      <c r="G52" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B53" s="19" t="s">
-        <v>122</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F53" s="20"/>
-      <c r="G53" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B54" s="19" t="s">
-        <v>124</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>125</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F54" s="20"/>
-      <c r="G54" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B55" s="19" t="s">
-        <v>126</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F55" s="20"/>
-      <c r="G55" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B56" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C56" s="19" t="s">
-        <v>129</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F56" s="20"/>
-      <c r="G56" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B57" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="C57" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F57" s="20"/>
-      <c r="G57" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B58" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="F58" s="20"/>
-      <c r="G58" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B59" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="C59" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E59" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="F59" s="20"/>
-      <c r="G59" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B60" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="C60" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="F60" s="20"/>
-      <c r="G60" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E61" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="F61" s="1"/>
-      <c r="G61" s="8" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G40" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="G2:G61">
+  <autoFilter ref="A1:G48" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="G2:G48">
     <cfRule type="cellIs" dxfId="1" priority="1" stopIfTrue="1" operator="equal">
       <formula>"Ja"</formula>
     </cfRule>
@@ -2770,12 +2447,24 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G2:G61" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G2:G48" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ja,Nein"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{11A4C3FC-25EB-4A5E-ADF7-5EA2FA0E0339}">
+          <x14:formula1>
+            <xm:f>Hilfstabellen!$A$2:$A$12</xm:f>
+          </x14:formula1>
+          <xm:sqref>F2:F48</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -2785,7 +2474,7 @@
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:H13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.5703125" style="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="61.5703125" style="10" bestFit="1" customWidth="1"/>
@@ -2796,191 +2485,191 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>140</v>
+        <v>99</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>142</v>
+        <v>101</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>143</v>
+        <v>102</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>144</v>
+        <v>103</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>145</v>
+        <v>104</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>147</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>148</v>
+        <v>107</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>149</v>
+        <v>108</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+        <v>109</v>
+      </c>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>151</v>
+        <v>110</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>152</v>
+        <v>111</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
+        <v>112</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
     </row>
     <row r="4" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>154</v>
+        <v>113</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>155</v>
+        <v>114</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
+        <v>115</v>
+      </c>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
     </row>
     <row r="5" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>157</v>
+        <v>116</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>158</v>
+        <v>117</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+        <v>118</v>
+      </c>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
     </row>
     <row r="6" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>160</v>
+        <v>119</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>161</v>
+        <v>120</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
+        <v>121</v>
+      </c>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>163</v>
+        <v>122</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>164</v>
+        <v>123</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
+        <v>124</v>
+      </c>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>167</v>
+        <v>126</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
+        <v>127</v>
+      </c>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>169</v>
+        <v>128</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>170</v>
+        <v>129</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>265</v>
-      </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
+        <v>130</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>172</v>
+        <v>131</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>173</v>
+        <v>132</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
+        <v>133</v>
+      </c>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="1:8" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>175</v>
+        <v>134</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>176</v>
+        <v>135</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
+        <v>136</v>
+      </c>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" s="11"/>
@@ -2999,7 +2688,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" style="10" customWidth="1"/>
     <col min="2" max="2" width="45.7109375" style="10" bestFit="1" customWidth="1"/>
@@ -3010,21 +2699,21 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>178</v>
+        <v>137</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>179</v>
+        <v>138</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>180</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C3" s="10" t="str">
         <f t="shared" ref="C3:C13" si="0">A3&amp;B3</f>
@@ -3033,10 +2722,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="C4" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3045,10 +2734,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C5" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3057,10 +2746,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>182</v>
+        <v>141</v>
       </c>
       <c r="C6" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3069,10 +2758,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>183</v>
+        <v>142</v>
       </c>
       <c r="C7" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3081,10 +2770,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="C8" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3093,10 +2782,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>184</v>
+        <v>143</v>
       </c>
       <c r="C9" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3105,10 +2794,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="C10" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3117,10 +2806,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>185</v>
+        <v>144</v>
       </c>
       <c r="C11" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3129,10 +2818,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>186</v>
+        <v>145</v>
       </c>
       <c r="C12" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3141,10 +2830,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>187</v>
+        <v>146</v>
       </c>
       <c r="C13" s="10" t="str">
         <f t="shared" si="0"/>
@@ -3160,7 +2849,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Tabelle2"/>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.42578125" bestFit="1" customWidth="1"/>
@@ -3169,1019 +2858,1066 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>179</v>
+        <v>138</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>188</v>
+        <v>147</v>
       </c>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>189</v>
+        <v>222</v>
       </c>
       <c r="D2" s="1" t="str">
-        <f t="shared" ref="D2:D22" si="0">LEFT(C2,FIND(" ",C2)-2)</f>
-        <v>Dentano</v>
+        <f t="shared" ref="D2" si="0">LEFT(C2,FIND(" ",C2)-2)</f>
+        <v>Behrends</v>
       </c>
       <c r="E2" s="1" t="str">
-        <f t="shared" ref="E2:E22" si="1">RIGHT(C2,LEN(C2)-FIND(" ",C2))</f>
-        <v>Melanie</v>
+        <f t="shared" ref="E2" si="1">RIGHT(C2,LEN(C2)-FIND(" ",C2))</f>
+        <v>Benjamin</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>185</v>
+        <v>144</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>190</v>
+        <v>164</v>
       </c>
       <c r="D3" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Förster</v>
+        <f t="shared" ref="D3:D27" si="2">LEFT(C3,FIND(" ",C3)-2)</f>
+        <v>Dammann</v>
       </c>
       <c r="E3" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Torsten</v>
+        <f t="shared" ref="E3:E27" si="3">RIGHT(C3,LEN(C3)-FIND(" ",C3))</f>
+        <v>Nils</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>191</v>
+        <v>148</v>
       </c>
       <c r="D4" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Gerdes</v>
+        <f t="shared" si="2"/>
+        <v>Dentano</v>
       </c>
       <c r="E4" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Simon Jakob</v>
+        <f t="shared" si="3"/>
+        <v>Melanie</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>187</v>
+        <v>146</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>192</v>
+        <v>149</v>
       </c>
       <c r="D5" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Grusche</v>
+        <f t="shared" si="2"/>
+        <v>Förster</v>
       </c>
       <c r="E5" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Sebastian</v>
+        <f t="shared" si="3"/>
+        <v>Torsten</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>182</v>
+        <v>141</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>193</v>
+        <v>150</v>
       </c>
       <c r="D6" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Höber</v>
+        <f t="shared" si="2"/>
+        <v>Gerdes</v>
       </c>
       <c r="E6" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Jennifer</v>
+        <f t="shared" si="3"/>
+        <v>Simon Jakob</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>183</v>
+        <v>142</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>194</v>
+        <v>151</v>
       </c>
       <c r="D7" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Lange</v>
+        <f t="shared" si="2"/>
+        <v>Grusche</v>
       </c>
       <c r="E7" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Yannik</v>
+        <f t="shared" si="3"/>
+        <v>Sebastian</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>195</v>
+        <v>152</v>
       </c>
       <c r="D8" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Marineße</v>
+        <f t="shared" si="2"/>
+        <v>Höber</v>
       </c>
       <c r="E8" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Loreen</v>
+        <f t="shared" si="3"/>
+        <v>Jennifer</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>184</v>
+        <v>143</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>196</v>
+        <v>223</v>
       </c>
       <c r="D9" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Meinke</v>
+        <f t="shared" si="2"/>
+        <v>Hoffmann</v>
       </c>
       <c r="E9" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Jannyn</v>
+        <f t="shared" si="3"/>
+        <v>Tobias</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>197</v>
+        <v>224</v>
       </c>
       <c r="D10" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Pendola</v>
+        <f t="shared" si="2"/>
+        <v>Klar-Janssen</v>
       </c>
       <c r="E10" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Christine</v>
+        <f t="shared" si="3"/>
+        <v>Markus</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>186</v>
+        <v>145</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>198</v>
+        <v>153</v>
       </c>
       <c r="D11" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Precht</v>
+        <f t="shared" si="2"/>
+        <v>Lange</v>
       </c>
       <c r="E11" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Maik</v>
+        <f t="shared" si="3"/>
+        <v>Yannik</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>199</v>
+        <v>225</v>
       </c>
       <c r="D12" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Reeck</v>
+        <f t="shared" si="2"/>
+        <v>Linnemann</v>
       </c>
       <c r="E12" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Torsten</v>
+        <f t="shared" si="3"/>
+        <v>Kristin</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
-        <v>200</v>
+        <v>154</v>
       </c>
       <c r="D13" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Riethmüller</v>
+        <f t="shared" si="2"/>
+        <v>Meinke</v>
       </c>
       <c r="E13" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Darron</v>
+        <f t="shared" si="3"/>
+        <v>Jannyn</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
-        <v>201</v>
+        <v>226</v>
       </c>
       <c r="D14" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Sasse</v>
+        <f t="shared" si="2"/>
+        <v>Mraw</v>
       </c>
       <c r="E14" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Corinna</v>
+        <f t="shared" si="3"/>
+        <v>Mohamed</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="s">
-        <v>202</v>
+        <v>155</v>
       </c>
       <c r="D15" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Sommer</v>
+        <f t="shared" si="2"/>
+        <v>Pendola</v>
       </c>
       <c r="E15" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Daniela</v>
+        <f t="shared" si="3"/>
+        <v>Christine</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C16" s="1" t="s">
-        <v>203</v>
+        <v>165</v>
       </c>
       <c r="D16" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Szodrowski</v>
+        <f t="shared" si="2"/>
+        <v>Pöppelmann</v>
       </c>
       <c r="E16" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Jakub</v>
+        <f t="shared" si="3"/>
+        <v>Manuela</v>
       </c>
     </row>
     <row r="17" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C17" s="1" t="s">
-        <v>204</v>
+        <v>156</v>
       </c>
       <c r="D17" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Wenke</v>
+        <f t="shared" si="2"/>
+        <v>Precht</v>
       </c>
       <c r="E17" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Franziska</v>
+        <f t="shared" si="3"/>
+        <v>Maik</v>
       </c>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C18" s="1" t="s">
-        <v>205</v>
+        <v>157</v>
       </c>
       <c r="D18" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Wolter</v>
+        <f t="shared" si="2"/>
+        <v>Reeck</v>
       </c>
       <c r="E18" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Sabine</v>
+        <f t="shared" si="3"/>
+        <v>Torsten</v>
       </c>
     </row>
     <row r="19" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C19" s="1" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="D19" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Zimmermann</v>
+        <f t="shared" si="2"/>
+        <v>Rosen</v>
       </c>
       <c r="E19" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Maike</v>
+        <f t="shared" si="3"/>
+        <v>Jennifer</v>
       </c>
     </row>
     <row r="20" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C20" s="1" t="s">
-        <v>207</v>
+        <v>158</v>
       </c>
       <c r="D20" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Dammann</v>
+        <f t="shared" si="2"/>
+        <v>Sasse</v>
       </c>
       <c r="E20" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Nils</v>
+        <f t="shared" si="3"/>
+        <v>Corinna</v>
       </c>
     </row>
     <row r="21" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C21" s="1" t="s">
-        <v>208</v>
+        <v>166</v>
       </c>
       <c r="D21" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Pöppelmann</v>
+        <f t="shared" si="2"/>
+        <v>Sauerwein</v>
       </c>
       <c r="E21" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Manuela</v>
+        <f t="shared" si="3"/>
+        <v>Swetlana</v>
       </c>
     </row>
     <row r="22" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C22" s="1" t="s">
-        <v>209</v>
+        <v>159</v>
       </c>
       <c r="D22" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Sauerwein</v>
+        <f t="shared" si="2"/>
+        <v>Sommer</v>
       </c>
       <c r="E22" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Swetlana</v>
+        <f t="shared" si="3"/>
+        <v>Daniela</v>
       </c>
     </row>
     <row r="23" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="C23" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D23" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>Szodrowski</v>
+      </c>
+      <c r="E23" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Jakub</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C24" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D24" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>Wenke</v>
+      </c>
+      <c r="E24" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Franziska</v>
+      </c>
+    </row>
+    <row r="25" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D25" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>Wolter</v>
+      </c>
+      <c r="E25" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Sabine</v>
+      </c>
     </row>
     <row r="26" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C26" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
+      <c r="C26" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="D26" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>Zimmermann</v>
+      </c>
+      <c r="E26" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Lara</v>
+      </c>
     </row>
     <row r="27" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C27" s="1" t="s">
-        <v>211</v>
+        <v>163</v>
       </c>
       <c r="D27" s="1" t="str">
-        <f t="shared" ref="D27:D48" si="2">LEFT(C27,FIND(" ",C27)-2)</f>
-        <v>Bönsch</v>
+        <f t="shared" si="2"/>
+        <v>Zimmermann</v>
       </c>
       <c r="E27" s="1" t="str">
-        <f t="shared" ref="E27:E48" si="3">RIGHT(C27,LEN(C27)-FIND(" ",C27))</f>
-        <v>Julia</v>
-      </c>
-    </row>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C28" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="D28" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Busko</v>
-      </c>
-      <c r="E28" s="1" t="str">
         <f t="shared" si="3"/>
-        <v>Nico</v>
-      </c>
-    </row>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C29" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D29" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Christians</v>
-      </c>
-      <c r="E29" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Yvonne</v>
+        <v>Maike</v>
       </c>
     </row>
     <row r="30" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C30" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="D30" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Dehnel</v>
-      </c>
-      <c r="E30" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Carola</v>
-      </c>
+      <c r="C30" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
     </row>
     <row r="31" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C31" s="1" t="s">
-        <v>215</v>
+        <v>168</v>
       </c>
       <c r="D31" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Döhren</v>
+        <f t="shared" ref="D31:D51" si="4">LEFT(C31,FIND(" ",C31)-2)</f>
+        <v>Bönsch</v>
       </c>
       <c r="E31" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Anna</v>
+        <f t="shared" ref="E31:E51" si="5">RIGHT(C31,LEN(C31)-FIND(" ",C31))</f>
+        <v>Julia</v>
       </c>
     </row>
     <row r="32" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
-        <v>216</v>
+        <v>169</v>
       </c>
       <c r="D32" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Freimuth</v>
+        <f t="shared" si="4"/>
+        <v>Christians</v>
       </c>
       <c r="E32" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Florian</v>
+        <f t="shared" si="5"/>
+        <v>Yvonne</v>
       </c>
     </row>
     <row r="33" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C33" s="1" t="s">
-        <v>217</v>
+        <v>170</v>
       </c>
       <c r="D33" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Hogelücht</v>
+        <f t="shared" si="4"/>
+        <v>Dehnel</v>
       </c>
       <c r="E33" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Pamela</v>
+        <f t="shared" si="5"/>
+        <v>Carola</v>
       </c>
     </row>
     <row r="34" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C34" s="1" t="s">
-        <v>218</v>
+        <v>171</v>
       </c>
       <c r="D34" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Hollatz</v>
+        <f t="shared" si="4"/>
+        <v>Döhren</v>
       </c>
       <c r="E34" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Jan-Helge</v>
+        <f t="shared" si="5"/>
+        <v>Anna</v>
       </c>
     </row>
     <row r="35" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C35" s="1" t="s">
-        <v>219</v>
+        <v>172</v>
       </c>
       <c r="D35" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Karagöz</v>
+        <f t="shared" si="4"/>
+        <v>Freimuth</v>
       </c>
       <c r="E35" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Irem</v>
+        <f t="shared" si="5"/>
+        <v>Florian</v>
       </c>
     </row>
     <row r="36" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C36" s="1" t="s">
-        <v>220</v>
+        <v>173</v>
       </c>
       <c r="D36" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Licher</v>
+        <f t="shared" si="4"/>
+        <v>Hogelücht</v>
       </c>
       <c r="E36" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Kea</v>
+        <f t="shared" si="5"/>
+        <v>Pamela</v>
       </c>
     </row>
     <row r="37" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C37" s="1" t="s">
-        <v>221</v>
+        <v>174</v>
       </c>
       <c r="D37" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Malinowski</v>
+        <f t="shared" si="4"/>
+        <v>Hollatz</v>
       </c>
       <c r="E37" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Bernd</v>
+        <f t="shared" si="5"/>
+        <v>Jan-Helge</v>
       </c>
     </row>
     <row r="38" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C38" s="1" t="s">
-        <v>222</v>
+        <v>175</v>
       </c>
       <c r="D38" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Marchwinski</v>
+        <f t="shared" si="4"/>
+        <v>Karagöz</v>
       </c>
       <c r="E38" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Kamil</v>
+        <f t="shared" si="5"/>
+        <v>Irem</v>
       </c>
     </row>
     <row r="39" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C39" s="1" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="D39" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Moritz</v>
+        <f t="shared" si="4"/>
+        <v>Licher</v>
       </c>
       <c r="E39" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Rayisa</v>
+        <f t="shared" si="5"/>
+        <v>Kea</v>
       </c>
     </row>
     <row r="40" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C40" s="1" t="s">
-        <v>224</v>
+        <v>177</v>
       </c>
       <c r="D40" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Muhle</v>
+        <f t="shared" si="4"/>
+        <v>Malinowski</v>
       </c>
       <c r="E40" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Britta</v>
+        <f t="shared" si="5"/>
+        <v>Bernd</v>
       </c>
     </row>
     <row r="41" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C41" s="1" t="s">
-        <v>225</v>
+        <v>178</v>
       </c>
       <c r="D41" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Münster</v>
+        <f t="shared" si="4"/>
+        <v>Marchwinski</v>
       </c>
       <c r="E41" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Stefan</v>
+        <f t="shared" si="5"/>
+        <v>Kamil</v>
       </c>
     </row>
     <row r="42" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C42" s="1" t="s">
-        <v>226</v>
+        <v>179</v>
       </c>
       <c r="D42" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Oelschläger</v>
+        <f t="shared" si="4"/>
+        <v>Moritz</v>
       </c>
       <c r="E42" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Gabriele</v>
+        <f t="shared" si="5"/>
+        <v>Rayisa</v>
       </c>
     </row>
     <row r="43" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C43" s="1" t="s">
-        <v>227</v>
+        <v>180</v>
       </c>
       <c r="D43" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Remmers</v>
+        <f t="shared" si="4"/>
+        <v>Muhle</v>
       </c>
       <c r="E43" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Liesa-Sofie</v>
+        <f t="shared" si="5"/>
+        <v>Britta</v>
       </c>
     </row>
     <row r="44" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C44" s="1" t="s">
-        <v>228</v>
+        <v>181</v>
       </c>
       <c r="D44" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Ritter</v>
+        <f t="shared" si="4"/>
+        <v>Münster</v>
       </c>
       <c r="E44" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Birgitt</v>
+        <f t="shared" si="5"/>
+        <v>Stefan</v>
       </c>
     </row>
     <row r="45" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C45" s="1" t="s">
-        <v>229</v>
+        <v>182</v>
       </c>
       <c r="D45" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Staroste</v>
+        <f t="shared" si="4"/>
+        <v>Oelschläger</v>
       </c>
       <c r="E45" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Heike</v>
+        <f t="shared" si="5"/>
+        <v>Gabriele</v>
       </c>
     </row>
     <row r="46" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C46" s="1" t="s">
-        <v>230</v>
+        <v>183</v>
       </c>
       <c r="D46" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Stening</v>
+        <f t="shared" si="4"/>
+        <v>Remmers</v>
       </c>
       <c r="E46" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Saskia</v>
+        <f t="shared" si="5"/>
+        <v>Liesa-Sofie</v>
       </c>
     </row>
     <row r="47" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C47" s="1" t="s">
-        <v>231</v>
+        <v>184</v>
       </c>
       <c r="D47" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Tensing</v>
+        <f t="shared" si="4"/>
+        <v>Ritter</v>
       </c>
       <c r="E47" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>Tobias</v>
+        <f t="shared" si="5"/>
+        <v>Birgitt</v>
       </c>
     </row>
     <row r="48" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C48" s="1" t="s">
-        <v>232</v>
+        <v>185</v>
       </c>
       <c r="D48" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
+        <v>Staroste</v>
+      </c>
+      <c r="E48" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Heike</v>
+      </c>
+    </row>
+    <row r="49" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C49" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D49" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Stening</v>
+      </c>
+      <c r="E49" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Saskia</v>
+      </c>
+    </row>
+    <row r="50" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C50" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D50" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>Tensing</v>
+      </c>
+      <c r="E50" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>Tobias</v>
+      </c>
+    </row>
+    <row r="51" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C51" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D51" s="1" t="str">
+        <f t="shared" si="4"/>
         <v>Widera</v>
       </c>
-      <c r="E48" s="1" t="str">
-        <f t="shared" si="3"/>
+      <c r="E51" s="1" t="str">
+        <f t="shared" si="5"/>
         <v>Hendrik</v>
       </c>
     </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C51" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="D51" s="4"/>
-      <c r="E51" s="4"/>
-    </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C52" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="D52" s="1" t="str">
-        <f t="shared" ref="D52:D69" si="4">LEFT(C52,FIND(" ",C52)-2)</f>
-        <v>Evers</v>
-      </c>
-      <c r="E52" s="1" t="str">
-        <f t="shared" ref="E52:E69" si="5">RIGHT(C52,LEN(C52)-FIND(" ",C52))</f>
-        <v>Marc William</v>
-      </c>
-    </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C53" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="D53" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Fluitman</v>
-      </c>
-      <c r="E53" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Jordan Bouke</v>
-      </c>
-    </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C54" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="D54" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Grummel</v>
-      </c>
-      <c r="E54" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Steffen</v>
-      </c>
+      <c r="C54" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
     </row>
     <row r="55" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C55" s="1" t="s">
-        <v>237</v>
+        <v>190</v>
       </c>
       <c r="D55" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Guida</v>
+        <f t="shared" ref="D55:D72" si="6">LEFT(C55,FIND(" ",C55)-2)</f>
+        <v>Evers</v>
       </c>
       <c r="E55" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Pasquale</v>
+        <f t="shared" ref="E55:E72" si="7">RIGHT(C55,LEN(C55)-FIND(" ",C55))</f>
+        <v>Marc William</v>
       </c>
     </row>
     <row r="56" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C56" s="1" t="s">
-        <v>238</v>
+        <v>191</v>
       </c>
       <c r="D56" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Kalyta</v>
+        <f t="shared" si="6"/>
+        <v>Fluitman</v>
       </c>
       <c r="E56" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Sonja</v>
+        <f t="shared" si="7"/>
+        <v>Jordan Bouke</v>
       </c>
     </row>
     <row r="57" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C57" s="1" t="s">
-        <v>239</v>
+        <v>192</v>
       </c>
       <c r="D57" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Kirmes</v>
+        <f t="shared" si="6"/>
+        <v>Grummel</v>
       </c>
       <c r="E57" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Manuela</v>
+        <f t="shared" si="7"/>
+        <v>Steffen</v>
       </c>
     </row>
     <row r="58" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C58" s="1" t="s">
-        <v>240</v>
+        <v>193</v>
       </c>
       <c r="D58" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Mücke</v>
+        <f t="shared" si="6"/>
+        <v>Guida</v>
       </c>
       <c r="E58" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Maik</v>
+        <f t="shared" si="7"/>
+        <v>Pasquale</v>
       </c>
     </row>
     <row r="59" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C59" s="1" t="s">
-        <v>241</v>
+        <v>194</v>
       </c>
       <c r="D59" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Ockenga</v>
+        <f t="shared" si="6"/>
+        <v>Kalyta</v>
       </c>
       <c r="E59" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Marco</v>
+        <f t="shared" si="7"/>
+        <v>Sonja</v>
       </c>
     </row>
     <row r="60" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C60" s="1" t="s">
-        <v>242</v>
+        <v>195</v>
       </c>
       <c r="D60" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Sandkötter</v>
+        <f t="shared" si="6"/>
+        <v>Kirmes</v>
       </c>
       <c r="E60" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Nicole</v>
+        <f t="shared" si="7"/>
+        <v>Manuela</v>
       </c>
     </row>
     <row r="61" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C61" s="1" t="s">
-        <v>243</v>
+        <v>196</v>
       </c>
       <c r="D61" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Seefeldt</v>
+        <f t="shared" si="6"/>
+        <v>Mücke</v>
       </c>
       <c r="E61" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Michelle Louisa</v>
+        <f t="shared" si="7"/>
+        <v>Maik</v>
       </c>
     </row>
     <row r="62" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C62" s="1" t="s">
-        <v>244</v>
+        <v>197</v>
       </c>
       <c r="D62" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Simke</v>
+        <f t="shared" si="6"/>
+        <v>Ockenga</v>
       </c>
       <c r="E62" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Katharina</v>
+        <f t="shared" si="7"/>
+        <v>Marco</v>
       </c>
     </row>
     <row r="63" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C63" s="1" t="s">
-        <v>245</v>
+        <v>198</v>
       </c>
       <c r="D63" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Stoll</v>
+        <f t="shared" si="6"/>
+        <v>Sandkötter</v>
       </c>
       <c r="E63" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Gustav</v>
+        <f t="shared" si="7"/>
+        <v>Nicole</v>
       </c>
     </row>
     <row r="64" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C64" s="1" t="s">
-        <v>246</v>
+        <v>199</v>
       </c>
       <c r="D64" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Süßmuth</v>
+        <f t="shared" si="6"/>
+        <v>Seefeldt</v>
       </c>
       <c r="E64" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Monika</v>
+        <f t="shared" si="7"/>
+        <v>Michelle Louisa</v>
       </c>
     </row>
     <row r="65" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C65" s="1" t="s">
-        <v>247</v>
+        <v>200</v>
       </c>
       <c r="D65" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Thiems</v>
+        <f t="shared" si="6"/>
+        <v>Simke</v>
       </c>
       <c r="E65" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Dennis</v>
+        <f t="shared" si="7"/>
+        <v>Katharina</v>
       </c>
     </row>
     <row r="66" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C66" s="1" t="s">
-        <v>248</v>
+        <v>201</v>
       </c>
       <c r="D66" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Hugen</v>
+        <f t="shared" si="6"/>
+        <v>Stoll</v>
       </c>
       <c r="E66" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Matthias</v>
+        <f t="shared" si="7"/>
+        <v>Gustav</v>
       </c>
     </row>
     <row r="67" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C67" s="1" t="s">
-        <v>249</v>
+        <v>202</v>
       </c>
       <c r="D67" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Duhm</v>
+        <f t="shared" si="6"/>
+        <v>Süßmuth</v>
       </c>
       <c r="E67" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Christina</v>
+        <f t="shared" si="7"/>
+        <v>Monika</v>
       </c>
     </row>
     <row r="68" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C68" s="1" t="s">
-        <v>250</v>
+        <v>203</v>
       </c>
       <c r="D68" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>Seldüz</v>
+        <f t="shared" si="6"/>
+        <v>Thiems</v>
       </c>
       <c r="E68" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>Selma</v>
+        <f t="shared" si="7"/>
+        <v>Dennis</v>
       </c>
     </row>
     <row r="69" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C69" s="1" t="s">
-        <v>251</v>
+        <v>204</v>
       </c>
       <c r="D69" s="1" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
+        <v>Hugen</v>
+      </c>
+      <c r="E69" s="1" t="str">
+        <f t="shared" si="7"/>
+        <v>Matthias</v>
+      </c>
+    </row>
+    <row r="70" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C70" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D70" s="1" t="str">
+        <f t="shared" si="6"/>
+        <v>Duhm</v>
+      </c>
+      <c r="E70" s="1" t="str">
+        <f t="shared" si="7"/>
+        <v>Christina</v>
+      </c>
+    </row>
+    <row r="71" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C71" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D71" s="1" t="str">
+        <f t="shared" si="6"/>
+        <v>Seldüz</v>
+      </c>
+      <c r="E71" s="1" t="str">
+        <f t="shared" si="7"/>
+        <v>Selma</v>
+      </c>
+    </row>
+    <row r="72" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C72" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D72" s="1" t="str">
+        <f t="shared" si="6"/>
         <v>Tangemann</v>
       </c>
-      <c r="E69" s="1" t="str">
-        <f t="shared" si="5"/>
+      <c r="E72" s="1" t="str">
+        <f t="shared" si="7"/>
         <v>Anne-Dörte</v>
       </c>
     </row>
-    <row r="72" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C72" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="D72" s="17"/>
-      <c r="E72" s="18"/>
-    </row>
-    <row r="73" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C73" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="D73" s="1" t="str">
-        <f t="shared" ref="D73:D84" si="6">LEFT(C73,FIND(" ",C73)-2)</f>
-        <v>Batschauer</v>
-      </c>
-      <c r="E73" s="1" t="str">
-        <f t="shared" ref="E73:E84" si="7">RIGHT(C73,LEN(C73)-FIND(" ",C73))</f>
-        <v>Vanessa</v>
-      </c>
-    </row>
-    <row r="74" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C74" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="D74" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Bodemer</v>
-      </c>
-      <c r="E74" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Raissa</v>
-      </c>
-    </row>
     <row r="75" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C75" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="D75" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Doberstein</v>
-      </c>
-      <c r="E75" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Vanessa</v>
-      </c>
+      <c r="C75" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D75" s="17"/>
+      <c r="E75" s="18"/>
     </row>
     <row r="76" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C76" s="1" t="s">
-        <v>256</v>
+        <v>209</v>
       </c>
       <c r="D76" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Fieberg</v>
+        <f t="shared" ref="D76:D87" si="8">LEFT(C76,FIND(" ",C76)-2)</f>
+        <v>Batschauer</v>
       </c>
       <c r="E76" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Kerstin</v>
+        <f t="shared" ref="E76:E87" si="9">RIGHT(C76,LEN(C76)-FIND(" ",C76))</f>
+        <v>Vanessa</v>
       </c>
     </row>
     <row r="77" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C77" s="1" t="s">
-        <v>257</v>
+        <v>210</v>
       </c>
       <c r="D77" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Kempf</v>
+        <f t="shared" si="8"/>
+        <v>Bodemer</v>
       </c>
       <c r="E77" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Cora</v>
+        <f t="shared" si="9"/>
+        <v>Raissa</v>
       </c>
     </row>
     <row r="78" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C78" s="1" t="s">
-        <v>258</v>
+        <v>211</v>
       </c>
       <c r="D78" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Kramer</v>
+        <f t="shared" si="8"/>
+        <v>Doberstein</v>
       </c>
       <c r="E78" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Angelika</v>
+        <f t="shared" si="9"/>
+        <v>Vanessa</v>
       </c>
     </row>
     <row r="79" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C79" s="1" t="s">
-        <v>259</v>
+        <v>212</v>
       </c>
       <c r="D79" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Kröger</v>
+        <f t="shared" si="8"/>
+        <v>Fieberg</v>
       </c>
       <c r="E79" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Markus</v>
+        <f t="shared" si="9"/>
+        <v>Kerstin</v>
       </c>
     </row>
     <row r="80" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C80" s="1" t="s">
-        <v>260</v>
+        <v>213</v>
       </c>
       <c r="D80" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Lübbe</v>
+        <f t="shared" si="8"/>
+        <v>Kempf</v>
       </c>
       <c r="E80" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Jens</v>
+        <f t="shared" si="9"/>
+        <v>Cora</v>
       </c>
     </row>
     <row r="81" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C81" s="1" t="s">
-        <v>261</v>
+        <v>214</v>
       </c>
       <c r="D81" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Pyka</v>
+        <f t="shared" si="8"/>
+        <v>Kramer</v>
       </c>
       <c r="E81" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Juliane Melanie</v>
+        <f t="shared" si="9"/>
+        <v>Angelika</v>
       </c>
     </row>
     <row r="82" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C82" s="1" t="s">
-        <v>262</v>
+        <v>215</v>
       </c>
       <c r="D82" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Rosenberg</v>
+        <f t="shared" si="8"/>
+        <v>Kröger</v>
       </c>
       <c r="E82" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Simone</v>
+        <f t="shared" si="9"/>
+        <v>Markus</v>
       </c>
     </row>
     <row r="83" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C83" s="1" t="s">
-        <v>263</v>
+        <v>216</v>
       </c>
       <c r="D83" s="1" t="str">
-        <f t="shared" si="6"/>
-        <v>Schmidt</v>
+        <f t="shared" si="8"/>
+        <v>Lübbe</v>
       </c>
       <c r="E83" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>Saskia</v>
+        <f t="shared" si="9"/>
+        <v>Jens</v>
       </c>
     </row>
     <row r="84" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C84" s="1" t="s">
-        <v>264</v>
+        <v>217</v>
       </c>
       <c r="D84" s="1" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
+        <v>Pyka</v>
+      </c>
+      <c r="E84" s="1" t="str">
+        <f t="shared" si="9"/>
+        <v>Juliane Melanie</v>
+      </c>
+    </row>
+    <row r="85" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C85" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D85" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Rosenberg</v>
+      </c>
+      <c r="E85" s="1" t="str">
+        <f t="shared" si="9"/>
+        <v>Simone</v>
+      </c>
+    </row>
+    <row r="86" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C86" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="D86" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Schmidt</v>
+      </c>
+      <c r="E86" s="1" t="str">
+        <f t="shared" si="9"/>
+        <v>Saskia</v>
+      </c>
+    </row>
+    <row r="87" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C87" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D87" s="1" t="str">
+        <f t="shared" si="8"/>
         <v>Terveer</v>
       </c>
-      <c r="E84" s="1" t="str">
-        <f t="shared" si="7"/>
+      <c r="E87" s="1" t="str">
+        <f t="shared" si="9"/>
         <v>Andrea</v>
       </c>
     </row>

</xml_diff>